<commit_message>
Review pass + level-up (iteration 2)
Make the model prescriptive, not just descriptive, and fix review findings:
- Goal-seek: cases needed for a target operating profit
- Capacity ceiling: max cases -> resulting revenue & profit
- Sensitivity tornado: which lever (price/volume/COGS/fixed/discounts) moves
  operating profit most at +/-10% (price dominates)
- Channel scorecard callout: most vs least profitable channel per case
- Fix waterfall: real dotted connector lines, hover tooltips, remove dead code
- Accessibility: aria-labels on channel inputs, SVG titles/roles, header tooltips
- engine.js gains goalSeek/capacity/sensitivity (headless-tested)
- Excel: matching Goal-Seek & Sensitivity sheet (now 7 sheets)
</commit_message>
<xml_diff>
--- a/revenue-forecast.xlsx
+++ b/revenue-forecast.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Profit Grid" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Monthly Plan" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Channel View" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Goal-Seek &amp; Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2781,4 +2782,265 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Goal-seek &amp; sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GOAL-SEEK — plan to a profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Target operating profit</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Cases needed</t>
+        </is>
+      </c>
+      <c r="B5" s="13">
+        <f>(B4+Model!$B$8)/Model!$B$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Gross revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="14">
+        <f>B5*Model!$B$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Net revenue</t>
+        </is>
+      </c>
+      <c r="B7" s="14">
+        <f>B5*Model!$B$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CAPACITY — what a ceiling delivers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Max cases you can sell</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Gross revenue</t>
+        </is>
+      </c>
+      <c r="B11" s="14">
+        <f>B10*Model!$B$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+      <c r="B12" s="14">
+        <f>B10*Model!$B$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Operating profit</t>
+        </is>
+      </c>
+      <c r="B13" s="27">
+        <f>B12-Model!$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — operating profit at ±10% (volumes held)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>−10%</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>+10%</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Swing</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Price / case</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,(Model!$B$13:$B$17*0.9)*(1-Model!$E$13:$E$17)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="C17" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,(Model!$B$13:$B$17*1.1)*(1-Model!$E$13:$E$17)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="D17" s="24">
+        <f>ABS(C17-B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Sales volume</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>Model!$B$27*0.9-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="C18" s="14">
+        <f>Model!$B$27*1.1-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="24">
+        <f>ABS(C18-B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>COGS / case</t>
+        </is>
+      </c>
+      <c r="B19" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,Model!$B$13:$B$17*(1-Model!$E$13:$E$17)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17*0.9)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="C19" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,Model!$B$13:$B$17*(1-Model!$E$13:$E$17)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17*1.1)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="D19" s="24">
+        <f>ABS(C19-B19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Fixed costs</t>
+        </is>
+      </c>
+      <c r="B20" s="14">
+        <f>Model!$B$27-Model!$B$8*0.9</f>
+        <v/>
+      </c>
+      <c r="C20" s="14">
+        <f>Model!$B$27-Model!$B$8*1.1</f>
+        <v/>
+      </c>
+      <c r="D20" s="24">
+        <f>ABS(C20-B20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Trade discounts</t>
+        </is>
+      </c>
+      <c r="B21" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,Model!$B$13:$B$17*(1-Model!$E$13:$E$17*0.9)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="C21" s="14">
+        <f>SUMPRODUCT(Model!$J$13:$J$17,Model!$B$13:$B$17*(1-Model!$E$13:$E$17*1.1)*(1-Model!$F$13:$F$17)-Model!$D$13:$D$17)-Model!$B$8</f>
+        <v/>
+      </c>
+      <c r="D21" s="24">
+        <f>ABS(C21-B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Longest swing = the lever that moves profit most. Price typically dominates.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>